<commit_message>
update status to trial-use 4430da51225fe24a20ec5dadf459134dbc0c0d44
</commit_message>
<xml_diff>
--- a/ig/nr-update-width/CodeSystem-fr-core-cs-circonstances-sortie.xlsx
+++ b/ig/nr-update-width/CodeSystem-fr-core-cs-circonstances-sortie.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.0</t>
+    <t>2.0.0-ballot</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-20T09:49:12+00:00</t>
+    <t>2024-02-20T10:34:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>